<commit_message>
1d cnn code 구현 및 feature selection 수정(5-fold)
</commit_message>
<xml_diff>
--- a/연구코드/results/regression/bmi_comparison_summary.xlsx
+++ b/연구코드/results/regression/bmi_comparison_summary.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
   <si>
     <t>Hospital</t>
   </si>
@@ -59,15 +59,12 @@
     <t>Log_Spec</t>
   </si>
   <si>
-    <t>TAMA_threshold</t>
+    <t>SMI_threshold</t>
   </si>
   <si>
     <t>강남</t>
   </si>
   <si>
-    <t>신촌</t>
-  </si>
-  <si>
     <t>C1_noBMI</t>
   </si>
   <si>
@@ -104,10 +101,7 @@
     <t>Case 4 (+BMI)</t>
   </si>
   <si>
-    <t>F:95.0/M:132.0</t>
-  </si>
-  <si>
-    <t>F:95.0/M:131.0</t>
+    <t>F:38.46/M:46.87</t>
   </si>
   <si>
     <t>Case_base</t>
@@ -501,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -556,10 +550,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -568,34 +562,34 @@
         <v>2</v>
       </c>
       <c r="F2">
-        <v>0.543</v>
+        <v>0.283</v>
       </c>
       <c r="G2">
-        <v>0.0401</v>
+        <v>0.0483</v>
       </c>
       <c r="H2">
-        <v>14.73</v>
+        <v>5.47</v>
       </c>
       <c r="I2">
-        <v>19.91</v>
+        <v>7.34</v>
       </c>
       <c r="J2">
-        <v>0.5992</v>
+        <v>0.4655</v>
       </c>
       <c r="K2">
-        <v>0.0403</v>
+        <v>0.023</v>
       </c>
       <c r="L2">
-        <v>0.7171999999999999</v>
+        <v>0.7311</v>
       </c>
       <c r="M2">
-        <v>0.3886</v>
+        <v>0.1434</v>
       </c>
       <c r="N2">
-        <v>0.8173</v>
+        <v>0.9267</v>
       </c>
       <c r="O2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -603,10 +597,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -615,34 +609,34 @@
         <v>3</v>
       </c>
       <c r="F3">
-        <v>0.662</v>
+        <v>0.4865</v>
       </c>
       <c r="G3">
-        <v>0.0367</v>
+        <v>0.0574</v>
       </c>
       <c r="H3">
-        <v>12.83</v>
+        <v>4.53</v>
       </c>
       <c r="I3">
-        <v>17.12</v>
+        <v>6.2</v>
       </c>
       <c r="J3">
-        <v>0.7427</v>
+        <v>0.7707000000000001</v>
       </c>
       <c r="K3">
-        <v>0.0188</v>
+        <v>0.0284</v>
       </c>
       <c r="L3">
-        <v>0.6762</v>
+        <v>0.6462</v>
       </c>
       <c r="M3">
-        <v>0.7647</v>
+        <v>0.8653</v>
       </c>
       <c r="N3">
-        <v>0.6491</v>
+        <v>0.5733</v>
       </c>
       <c r="O3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -650,10 +644,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -662,34 +656,34 @@
         <v>6</v>
       </c>
       <c r="F4">
-        <v>0.63</v>
+        <v>0.4089</v>
       </c>
       <c r="G4">
-        <v>0.0407</v>
+        <v>0.0456</v>
       </c>
       <c r="H4">
-        <v>13.22</v>
+        <v>4.97</v>
       </c>
       <c r="I4">
-        <v>17.91</v>
+        <v>6.66</v>
       </c>
       <c r="J4">
-        <v>0.7</v>
+        <v>0.6813</v>
       </c>
       <c r="K4">
-        <v>0.0276</v>
+        <v>0.0203</v>
       </c>
       <c r="L4">
-        <v>0.6198</v>
+        <v>0.6095</v>
       </c>
       <c r="M4">
-        <v>0.7741</v>
+        <v>0.7569</v>
       </c>
       <c r="N4">
-        <v>0.5726</v>
+        <v>0.5606</v>
       </c>
       <c r="O4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -697,10 +691,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -709,34 +703,34 @@
         <v>7</v>
       </c>
       <c r="F5">
-        <v>0.678</v>
+        <v>0.4997</v>
       </c>
       <c r="G5">
-        <v>0.0357</v>
+        <v>0.051</v>
       </c>
       <c r="H5">
-        <v>12.53</v>
+        <v>4.48</v>
       </c>
       <c r="I5">
-        <v>16.71</v>
+        <v>6.13</v>
       </c>
       <c r="J5">
-        <v>0.751</v>
+        <v>0.7715</v>
       </c>
       <c r="K5">
-        <v>0.0227</v>
+        <v>0.029</v>
       </c>
       <c r="L5">
-        <v>0.7004</v>
+        <v>0.7062</v>
       </c>
       <c r="M5">
-        <v>0.7393999999999999</v>
+        <v>0.7479</v>
       </c>
       <c r="N5">
-        <v>0.6883</v>
+        <v>0.6924</v>
       </c>
       <c r="O5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -744,10 +738,10 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -756,34 +750,34 @@
         <v>45</v>
       </c>
       <c r="F6">
-        <v>0.621</v>
+        <v>0.3891</v>
       </c>
       <c r="G6">
-        <v>0.0339</v>
+        <v>0.0445</v>
       </c>
       <c r="H6">
-        <v>13.39</v>
+        <v>5.03</v>
       </c>
       <c r="I6">
-        <v>18.13</v>
+        <v>6.77</v>
       </c>
       <c r="J6">
-        <v>0.7104</v>
+        <v>0.6839</v>
       </c>
       <c r="K6">
-        <v>0.026</v>
+        <v>0.0356</v>
       </c>
       <c r="L6">
-        <v>0.6344</v>
+        <v>0.6403</v>
       </c>
       <c r="M6">
-        <v>0.7834</v>
+        <v>0.7246</v>
       </c>
       <c r="N6">
-        <v>0.5889</v>
+        <v>0.6123</v>
       </c>
       <c r="O6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -791,10 +785,10 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -803,316 +797,34 @@
         <v>46</v>
       </c>
       <c r="F7">
-        <v>0.6682</v>
+        <v>0.4831</v>
       </c>
       <c r="G7">
-        <v>0.0318</v>
+        <v>0.0543</v>
       </c>
       <c r="H7">
-        <v>12.77</v>
+        <v>4.57</v>
       </c>
       <c r="I7">
-        <v>16.96</v>
+        <v>6.23</v>
       </c>
       <c r="J7">
-        <v>0.74</v>
+        <v>0.7589</v>
       </c>
       <c r="K7">
-        <v>0.0287</v>
+        <v>0.0397</v>
       </c>
       <c r="L7">
-        <v>0.6674</v>
+        <v>0.6864</v>
       </c>
       <c r="M7">
-        <v>0.7834</v>
+        <v>0.7716</v>
       </c>
       <c r="N7">
-        <v>0.6319</v>
+        <v>0.6582</v>
       </c>
       <c r="O7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="b">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8">
-        <v>0.5216</v>
-      </c>
-      <c r="G8">
-        <v>0.06560000000000001</v>
-      </c>
-      <c r="H8">
-        <v>15.94</v>
-      </c>
-      <c r="I8">
-        <v>21.24</v>
-      </c>
-      <c r="J8">
-        <v>0.6076</v>
-      </c>
-      <c r="K8">
-        <v>0.0299</v>
-      </c>
-      <c r="L8">
-        <v>0.6588000000000001</v>
-      </c>
-      <c r="M8">
-        <v>0.5505</v>
-      </c>
-      <c r="N8">
-        <v>0.6938</v>
-      </c>
-      <c r="O8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
-      </c>
-      <c r="F9">
-        <v>0.6398</v>
-      </c>
-      <c r="G9">
-        <v>0.0629</v>
-      </c>
-      <c r="H9">
-        <v>13.82</v>
-      </c>
-      <c r="I9">
-        <v>18.42</v>
-      </c>
-      <c r="J9">
-        <v>0.7513</v>
-      </c>
-      <c r="K9">
-        <v>0.0332</v>
-      </c>
-      <c r="L9">
-        <v>0.6541</v>
-      </c>
-      <c r="M9">
-        <v>0.7988</v>
-      </c>
-      <c r="N9">
-        <v>0.6073</v>
-      </c>
-      <c r="O9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>6</v>
-      </c>
-      <c r="F10">
-        <v>0.5444</v>
-      </c>
-      <c r="G10">
-        <v>0.0587</v>
-      </c>
-      <c r="H10">
-        <v>15.56</v>
-      </c>
-      <c r="I10">
-        <v>20.73</v>
-      </c>
-      <c r="J10">
-        <v>0.6441</v>
-      </c>
-      <c r="K10">
-        <v>0.043</v>
-      </c>
-      <c r="L10">
-        <v>0.6446</v>
-      </c>
-      <c r="M10">
-        <v>0.6114000000000001</v>
-      </c>
-      <c r="N10">
-        <v>0.6552</v>
-      </c>
-      <c r="O10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" t="b">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>7</v>
-      </c>
-      <c r="F11">
-        <v>0.6415</v>
-      </c>
-      <c r="G11">
-        <v>0.0615</v>
-      </c>
-      <c r="H11">
-        <v>13.83</v>
-      </c>
-      <c r="I11">
-        <v>18.37</v>
-      </c>
-      <c r="J11">
-        <v>0.7502</v>
-      </c>
-      <c r="K11">
-        <v>0.0362</v>
-      </c>
-      <c r="L11">
-        <v>0.6596</v>
-      </c>
-      <c r="M11">
-        <v>0.8055</v>
-      </c>
-      <c r="N11">
-        <v>0.6125</v>
-      </c>
-      <c r="O11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>58</v>
-      </c>
-      <c r="F12">
-        <v>0.535</v>
-      </c>
-      <c r="G12">
-        <v>0.0693</v>
-      </c>
-      <c r="H12">
-        <v>15.47</v>
-      </c>
-      <c r="I12">
-        <v>20.92</v>
-      </c>
-      <c r="J12">
-        <v>0.6784</v>
-      </c>
-      <c r="K12">
-        <v>0.0236</v>
-      </c>
-      <c r="L12">
-        <v>0.6657999999999999</v>
-      </c>
-      <c r="M12">
-        <v>0.641</v>
-      </c>
-      <c r="N12">
-        <v>0.674</v>
-      </c>
-      <c r="O12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" t="s">
         <v>28</v>
-      </c>
-      <c r="D13" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <v>59</v>
-      </c>
-      <c r="F13">
-        <v>0.634</v>
-      </c>
-      <c r="G13">
-        <v>0.059</v>
-      </c>
-      <c r="H13">
-        <v>14</v>
-      </c>
-      <c r="I13">
-        <v>18.56</v>
-      </c>
-      <c r="J13">
-        <v>0.7529</v>
-      </c>
-      <c r="K13">
-        <v>0.0321</v>
-      </c>
-      <c r="L13">
-        <v>0.7060999999999999</v>
-      </c>
-      <c r="M13">
-        <v>0.7572</v>
-      </c>
-      <c r="N13">
-        <v>0.6896</v>
-      </c>
-      <c r="O13" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1122,7 +834,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1130,31 +842,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -1162,31 +874,31 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2">
-        <v>0.119</v>
+        <v>0.2035</v>
       </c>
       <c r="D2">
-        <v>-2.79</v>
+        <v>-1.14</v>
       </c>
       <c r="E2">
-        <v>0.1435</v>
+        <v>0.3052</v>
       </c>
       <c r="F2">
-        <v>-0.041</v>
+        <v>-0.0849</v>
       </c>
       <c r="G2">
-        <v>0.543</v>
+        <v>0.283</v>
       </c>
       <c r="H2">
-        <v>0.662</v>
+        <v>0.4865</v>
       </c>
       <c r="I2">
-        <v>0.5992</v>
+        <v>0.4655</v>
       </c>
       <c r="J2">
-        <v>0.7427</v>
+        <v>0.7707000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1194,31 +906,31 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C3">
-        <v>0.048</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="D3">
-        <v>-1.2</v>
+        <v>-0.53</v>
       </c>
       <c r="E3">
-        <v>0.051</v>
+        <v>0.0902</v>
       </c>
       <c r="F3">
-        <v>0.0806</v>
+        <v>0.09669999999999999</v>
       </c>
       <c r="G3">
-        <v>0.63</v>
+        <v>0.4089</v>
       </c>
       <c r="H3">
-        <v>0.678</v>
+        <v>0.4997</v>
       </c>
       <c r="I3">
-        <v>0.7</v>
+        <v>0.6813</v>
       </c>
       <c r="J3">
-        <v>0.751</v>
+        <v>0.7715</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1226,127 +938,31 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C4">
-        <v>0.0472</v>
+        <v>0.094</v>
       </c>
       <c r="D4">
-        <v>-1.17</v>
+        <v>-0.54</v>
       </c>
       <c r="E4">
-        <v>0.0296</v>
+        <v>0.075</v>
       </c>
       <c r="F4">
-        <v>0.033</v>
+        <v>0.0461</v>
       </c>
       <c r="G4">
-        <v>0.621</v>
+        <v>0.3891</v>
       </c>
       <c r="H4">
-        <v>0.6682</v>
+        <v>0.4831</v>
       </c>
       <c r="I4">
-        <v>0.7104</v>
+        <v>0.6839</v>
       </c>
       <c r="J4">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5">
-        <v>0.1182</v>
-      </c>
-      <c r="D5">
-        <v>-2.82</v>
-      </c>
-      <c r="E5">
-        <v>0.1437</v>
-      </c>
-      <c r="F5">
-        <v>-0.0047</v>
-      </c>
-      <c r="G5">
-        <v>0.5216</v>
-      </c>
-      <c r="H5">
-        <v>0.6398</v>
-      </c>
-      <c r="I5">
-        <v>0.6076</v>
-      </c>
-      <c r="J5">
-        <v>0.7513</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6">
-        <v>0.09710000000000001</v>
-      </c>
-      <c r="D6">
-        <v>-2.36</v>
-      </c>
-      <c r="E6">
-        <v>0.1061</v>
-      </c>
-      <c r="F6">
-        <v>0.015</v>
-      </c>
-      <c r="G6">
-        <v>0.5444</v>
-      </c>
-      <c r="H6">
-        <v>0.6415</v>
-      </c>
-      <c r="I6">
-        <v>0.6441</v>
-      </c>
-      <c r="J6">
-        <v>0.7502</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7">
-        <v>0.099</v>
-      </c>
-      <c r="D7">
-        <v>-2.36</v>
-      </c>
-      <c r="E7">
-        <v>0.0745</v>
-      </c>
-      <c r="F7">
-        <v>0.0403</v>
-      </c>
-      <c r="G7">
-        <v>0.535</v>
-      </c>
-      <c r="H7">
-        <v>0.634</v>
-      </c>
-      <c r="I7">
-        <v>0.6784</v>
-      </c>
-      <c r="J7">
-        <v>0.7529</v>
+        <v>0.7589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>